<commit_message>
Keep Term-Months rows as line items in Software Only (PDF + XLSX)
Sales ops needs the Term-Months filler row carried through to the
downstream CRM. Both Software Only parsers previously discarded it as
a sub-header that repeats after every real line item.

Emit a LineItem per source occurrence with Vpn="Term-Months",
Description="Term in months", Term and Qty set to the source term
value, and Cost=Msrp=0m. ForeignUpliftWriter's existing NonZeroPrice
helper renders the zero prices as the 0.000001 sentinel the uplift
app requires.

Golden fixtures regenerated for XQ-4076249, XQ-4157308 and
XQ-4165884. Spec docs and AGENTS.md updated (Hardware Only no longer
contrasts with Software Only on this rule). Validation totals
unchanged because zero-cost rows contribute nothing to the sum.
</commit_message>
<xml_diff>
--- a/samples/outputs/XQ-4076249_parsed.xlsx
+++ b/samples/outputs/XQ-4076249_parsed.xlsx
@@ -115,6 +115,12 @@
   </x:si>
   <x:si>
     <x:t>USD</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Term-Months</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Term in months</x:t>
   </x:si>
   <x:si>
     <x:t>SW-NCI-PRO-PR</x:t>
@@ -493,7 +499,7 @@
   <x:sheetPr>
     <x:outlinePr summaryBelow="1" summaryRight="1"/>
   </x:sheetPr>
-  <x:dimension ref="A1:AA8"/>
+  <x:dimension ref="A1:AA13"/>
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:sheetData>
     <x:row r="1" spans="1:27">
@@ -633,7 +639,7 @@
         <x:v>34</x:v>
       </x:c>
       <x:c r="F4" s="0">
-        <x:v>864</x:v>
+        <x:v>60</x:v>
       </x:c>
       <x:c r="K4" s="0">
         <x:v>5</x:v>
@@ -645,10 +651,10 @@
         <x:v>32</x:v>
       </x:c>
       <x:c r="T4" s="0">
-        <x:v>600.6</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="U4" s="0">
-        <x:v>2275</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="V4" s="0">
         <x:v>1</x:v>
@@ -662,13 +668,13 @@
         <x:v>28</x:v>
       </x:c>
       <x:c r="D5" s="0" t="s">
-        <x:v>33</x:v>
+        <x:v>35</x:v>
       </x:c>
       <x:c r="E5" s="0" t="s">
-        <x:v>34</x:v>
+        <x:v>36</x:v>
       </x:c>
       <x:c r="F5" s="0">
-        <x:v>1232</x:v>
+        <x:v>864</x:v>
       </x:c>
       <x:c r="K5" s="0">
         <x:v>5</x:v>
@@ -697,13 +703,13 @@
         <x:v>28</x:v>
       </x:c>
       <x:c r="D6" s="0" t="s">
-        <x:v>35</x:v>
+        <x:v>33</x:v>
       </x:c>
       <x:c r="E6" s="0" t="s">
-        <x:v>36</x:v>
+        <x:v>34</x:v>
       </x:c>
       <x:c r="F6" s="0">
-        <x:v>145</x:v>
+        <x:v>60</x:v>
       </x:c>
       <x:c r="K6" s="0">
         <x:v>5</x:v>
@@ -715,10 +721,10 @@
         <x:v>32</x:v>
       </x:c>
       <x:c r="T6" s="0">
-        <x:v>912.12</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="U6" s="0">
-        <x:v>3455</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="V6" s="0">
         <x:v>1</x:v>
@@ -732,13 +738,13 @@
         <x:v>28</x:v>
       </x:c>
       <x:c r="D7" s="0" t="s">
-        <x:v>37</x:v>
+        <x:v>35</x:v>
       </x:c>
       <x:c r="E7" s="0" t="s">
-        <x:v>38</x:v>
+        <x:v>36</x:v>
       </x:c>
       <x:c r="F7" s="0">
-        <x:v>145</x:v>
+        <x:v>1232</x:v>
       </x:c>
       <x:c r="K7" s="0">
         <x:v>5</x:v>
@@ -750,21 +756,196 @@
         <x:v>32</x:v>
       </x:c>
       <x:c r="T7" s="0">
+        <x:v>600.6</x:v>
+      </x:c>
+      <x:c r="U7" s="0">
+        <x:v>2275</x:v>
+      </x:c>
+      <x:c r="V7" s="0">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8" spans="1:27">
+      <x:c r="A8" s="0">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="B8" s="0" t="s">
+        <x:v>28</x:v>
+      </x:c>
+      <x:c r="D8" s="0" t="s">
+        <x:v>33</x:v>
+      </x:c>
+      <x:c r="E8" s="0" t="s">
+        <x:v>34</x:v>
+      </x:c>
+      <x:c r="F8" s="0">
+        <x:v>60</x:v>
+      </x:c>
+      <x:c r="K8" s="0">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="R8" s="0" t="s">
+        <x:v>31</x:v>
+      </x:c>
+      <x:c r="S8" s="0" t="s">
+        <x:v>32</x:v>
+      </x:c>
+      <x:c r="T8" s="0">
+        <x:v>1E-06</x:v>
+      </x:c>
+      <x:c r="U8" s="0">
+        <x:v>1E-06</x:v>
+      </x:c>
+      <x:c r="V8" s="0">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9" spans="1:27">
+      <x:c r="A9" s="0">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="B9" s="0" t="s">
+        <x:v>28</x:v>
+      </x:c>
+      <x:c r="D9" s="0" t="s">
+        <x:v>37</x:v>
+      </x:c>
+      <x:c r="E9" s="0" t="s">
+        <x:v>38</x:v>
+      </x:c>
+      <x:c r="F9" s="0">
+        <x:v>145</x:v>
+      </x:c>
+      <x:c r="K9" s="0">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="R9" s="0" t="s">
+        <x:v>31</x:v>
+      </x:c>
+      <x:c r="S9" s="0" t="s">
+        <x:v>32</x:v>
+      </x:c>
+      <x:c r="T9" s="0">
+        <x:v>912.12</x:v>
+      </x:c>
+      <x:c r="U9" s="0">
+        <x:v>3455</x:v>
+      </x:c>
+      <x:c r="V9" s="0">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10" spans="1:27">
+      <x:c r="A10" s="0">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="B10" s="0" t="s">
+        <x:v>28</x:v>
+      </x:c>
+      <x:c r="D10" s="0" t="s">
+        <x:v>33</x:v>
+      </x:c>
+      <x:c r="E10" s="0" t="s">
+        <x:v>34</x:v>
+      </x:c>
+      <x:c r="F10" s="0">
+        <x:v>60</x:v>
+      </x:c>
+      <x:c r="K10" s="0">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="R10" s="0" t="s">
+        <x:v>31</x:v>
+      </x:c>
+      <x:c r="S10" s="0" t="s">
+        <x:v>32</x:v>
+      </x:c>
+      <x:c r="T10" s="0">
+        <x:v>1E-06</x:v>
+      </x:c>
+      <x:c r="U10" s="0">
+        <x:v>1E-06</x:v>
+      </x:c>
+      <x:c r="V10" s="0">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11" spans="1:27">
+      <x:c r="A11" s="0">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="B11" s="0" t="s">
+        <x:v>28</x:v>
+      </x:c>
+      <x:c r="D11" s="0" t="s">
+        <x:v>39</x:v>
+      </x:c>
+      <x:c r="E11" s="0" t="s">
+        <x:v>40</x:v>
+      </x:c>
+      <x:c r="F11" s="0">
+        <x:v>145</x:v>
+      </x:c>
+      <x:c r="K11" s="0">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="R11" s="0" t="s">
+        <x:v>31</x:v>
+      </x:c>
+      <x:c r="S11" s="0" t="s">
+        <x:v>32</x:v>
+      </x:c>
+      <x:c r="T11" s="0">
         <x:v>153.91</x:v>
       </x:c>
-      <x:c r="U7" s="0">
+      <x:c r="U11" s="0">
         <x:v>583</x:v>
       </x:c>
-      <x:c r="V7" s="0">
-        <x:v>1</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="8" spans="1:27">
-      <x:c r="B8" s="0" t="s">
-        <x:v>39</x:v>
-      </x:c>
-      <x:c r="D8" s="0" t="s">
-        <x:v>40</x:v>
+      <x:c r="V11" s="0">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12" spans="1:27">
+      <x:c r="A12" s="0">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="B12" s="0" t="s">
+        <x:v>28</x:v>
+      </x:c>
+      <x:c r="D12" s="0" t="s">
+        <x:v>33</x:v>
+      </x:c>
+      <x:c r="E12" s="0" t="s">
+        <x:v>34</x:v>
+      </x:c>
+      <x:c r="F12" s="0">
+        <x:v>60</x:v>
+      </x:c>
+      <x:c r="K12" s="0">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="R12" s="0" t="s">
+        <x:v>31</x:v>
+      </x:c>
+      <x:c r="S12" s="0" t="s">
+        <x:v>32</x:v>
+      </x:c>
+      <x:c r="T12" s="0">
+        <x:v>1E-06</x:v>
+      </x:c>
+      <x:c r="U12" s="0">
+        <x:v>1E-06</x:v>
+      </x:c>
+      <x:c r="V12" s="0">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13" spans="1:27">
+      <x:c r="B13" s="0" t="s">
+        <x:v>41</x:v>
+      </x:c>
+      <x:c r="D13" s="0" t="s">
+        <x:v>42</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>